<commit_message>
#228 EXCEL rebase bug fix
</commit_message>
<xml_diff>
--- a/Sources/Cuga-Calibration-Solution/Assets/Data/InitData.xlsx
+++ b/Sources/Cuga-Calibration-Solution/Assets/Data/InitData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\Code\CSharp\semix\xuankaizhi\netcore_semix_cuga_calibration\Sources\Cuga-Calibration-Solution\Assets\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF94D977-196D-43DB-85BF-C910A4EE969D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A88E05B-D443-4BF4-B2C7-BC7DD2CCBF76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="456" uniqueCount="201">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="464" uniqueCount="205">
   <si>
     <t>Id</t>
   </si>
@@ -705,6 +705,18 @@
   <si>
     <t>CugaCalibration.ViewModels.Common.Windows.Tools.AODWaveform.ChirpAODWaveformElectrodeDelayWindowViewModel</t>
     <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>Side Channel Flexible Aperture</t>
+  </si>
+  <si>
+    <t>CugaCalibration.ViewModels.Fourier.FourierSideChannelFlexibleApertureViewModel</t>
+  </si>
+  <si>
+    <t>Side Channel Specular Blocker</t>
+  </si>
+  <si>
+    <t>CugaCalibration.ViewModels.Fourier.FourierSideChannelSpecularBlockerViewModel</t>
   </si>
 </sst>
 </file>
@@ -3426,7 +3438,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:I93"/>
+  <dimension ref="A1:I95"/>
   <sheetFormatPr defaultColWidth="19.75" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19.75" style="1"/>
@@ -4700,308 +4712,310 @@
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A52" s="3">
-        <v>2</v>
-      </c>
-      <c r="B52" s="4" t="s">
-        <v>127</v>
+        <v>1902</v>
+      </c>
+      <c r="B52" s="6" t="s">
+        <v>201</v>
       </c>
       <c r="C52" s="3">
-        <v>-1</v>
+        <v>19</v>
       </c>
       <c r="D52" s="3">
-        <v>2</v>
+        <v>1902</v>
       </c>
       <c r="E52" s="3"/>
       <c r="F52" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="G52" s="4"/>
+        <v>39</v>
+      </c>
+      <c r="G52" s="6" t="s">
+        <v>202</v>
+      </c>
       <c r="H52" s="4"/>
-      <c r="I52" s="4" t="s">
-        <v>127</v>
+      <c r="I52" s="6" t="s">
+        <v>201</v>
       </c>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A53" s="3">
-        <v>21</v>
-      </c>
-      <c r="B53" s="4" t="s">
-        <v>128</v>
+        <v>1903</v>
+      </c>
+      <c r="B53" s="6" t="s">
+        <v>203</v>
       </c>
       <c r="C53" s="3">
-        <v>2</v>
+        <v>19</v>
       </c>
       <c r="D53" s="3">
-        <v>21</v>
+        <v>1903</v>
       </c>
       <c r="E53" s="3"/>
       <c r="F53" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="G53" s="4"/>
+        <v>39</v>
+      </c>
+      <c r="G53" s="6" t="s">
+        <v>204</v>
+      </c>
       <c r="H53" s="4"/>
-      <c r="I53" s="4" t="s">
-        <v>128</v>
+      <c r="I53" s="6" t="s">
+        <v>203</v>
       </c>
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A54" s="3">
-        <v>2110</v>
+        <v>2</v>
       </c>
       <c r="B54" s="4" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="C54" s="3">
-        <v>21</v>
+        <v>-1</v>
       </c>
       <c r="D54" s="3">
-        <v>2110</v>
+        <v>2</v>
       </c>
       <c r="E54" s="3"/>
       <c r="F54" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="G54" s="4" t="s">
-        <v>130</v>
-      </c>
+        <v>36</v>
+      </c>
+      <c r="G54" s="4"/>
       <c r="H54" s="4"/>
       <c r="I54" s="4" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A55" s="3">
-        <v>2111</v>
+        <v>21</v>
       </c>
       <c r="B55" s="4" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="C55" s="3">
+        <v>2</v>
+      </c>
+      <c r="D55" s="3">
         <v>21</v>
-      </c>
-      <c r="D55" s="3">
-        <v>2111</v>
       </c>
       <c r="E55" s="3"/>
       <c r="F55" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="G55" s="4" t="s">
-        <v>132</v>
-      </c>
+        <v>36</v>
+      </c>
+      <c r="G55" s="4"/>
       <c r="H55" s="4"/>
       <c r="I55" s="4" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A56" s="3">
-        <v>2112</v>
+        <v>2110</v>
       </c>
       <c r="B56" s="4" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="C56" s="3">
         <v>21</v>
       </c>
       <c r="D56" s="3">
-        <v>2112</v>
+        <v>2110</v>
       </c>
       <c r="E56" s="3"/>
       <c r="F56" s="3" t="s">
         <v>39</v>
       </c>
       <c r="G56" s="4" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="H56" s="4"/>
       <c r="I56" s="4" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A57" s="3">
-        <v>2113</v>
+        <v>2111</v>
       </c>
       <c r="B57" s="4" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C57" s="3">
         <v>21</v>
       </c>
       <c r="D57" s="3">
-        <v>2113</v>
+        <v>2111</v>
       </c>
       <c r="E57" s="3"/>
       <c r="F57" s="3" t="s">
         <v>39</v>
       </c>
       <c r="G57" s="4" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="H57" s="4"/>
       <c r="I57" s="4" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A58" s="3">
-        <v>22</v>
+        <v>2112</v>
       </c>
       <c r="B58" s="4" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="C58" s="3">
-        <v>2</v>
+        <v>21</v>
       </c>
       <c r="D58" s="3">
-        <v>22</v>
+        <v>2112</v>
       </c>
       <c r="E58" s="3"/>
       <c r="F58" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="G58" s="4"/>
+        <v>39</v>
+      </c>
+      <c r="G58" s="4" t="s">
+        <v>134</v>
+      </c>
       <c r="H58" s="4"/>
       <c r="I58" s="4" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A59" s="3">
-        <v>2201</v>
+        <v>2113</v>
       </c>
       <c r="B59" s="4" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="C59" s="3">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D59" s="3">
-        <v>2201</v>
+        <v>2113</v>
       </c>
       <c r="E59" s="3"/>
       <c r="F59" s="3" t="s">
         <v>39</v>
       </c>
       <c r="G59" s="4" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="H59" s="4"/>
       <c r="I59" s="4" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A60" s="3">
-        <v>2202</v>
+        <v>22</v>
       </c>
       <c r="B60" s="4" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="C60" s="3">
+        <v>2</v>
+      </c>
+      <c r="D60" s="3">
         <v>22</v>
-      </c>
-      <c r="D60" s="3">
-        <v>2202</v>
       </c>
       <c r="E60" s="3"/>
       <c r="F60" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="G60" s="4" t="s">
-        <v>140</v>
-      </c>
+        <v>36</v>
+      </c>
+      <c r="G60" s="4"/>
       <c r="H60" s="4"/>
       <c r="I60" s="4" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A61" s="3">
-        <v>2203</v>
+        <v>2201</v>
       </c>
       <c r="B61" s="4" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="C61" s="3">
         <v>22</v>
       </c>
       <c r="D61" s="3">
-        <v>2203</v>
+        <v>2201</v>
       </c>
       <c r="E61" s="3"/>
       <c r="F61" s="3" t="s">
         <v>39</v>
       </c>
       <c r="G61" s="4" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="H61" s="4"/>
       <c r="I61" s="4" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A62" s="3">
-        <v>23</v>
+        <v>2202</v>
       </c>
       <c r="B62" s="4" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="C62" s="3">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D62" s="3">
-        <v>23</v>
+        <v>2202</v>
       </c>
       <c r="E62" s="3"/>
       <c r="F62" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="G62" s="4"/>
+        <v>39</v>
+      </c>
+      <c r="G62" s="4" t="s">
+        <v>140</v>
+      </c>
       <c r="H62" s="4"/>
       <c r="I62" s="4" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A63" s="3">
-        <v>2301</v>
+        <v>2203</v>
       </c>
       <c r="B63" s="4" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="C63" s="3">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D63" s="3">
-        <v>2301</v>
+        <v>2203</v>
       </c>
       <c r="E63" s="3"/>
       <c r="F63" s="3" t="s">
         <v>39</v>
       </c>
       <c r="G63" s="4" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="H63" s="4"/>
       <c r="I63" s="4" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A64" s="3">
-        <v>2302</v>
+        <v>23</v>
       </c>
       <c r="B64" s="4" t="s">
-        <v>75</v>
+        <v>143</v>
       </c>
       <c r="C64" s="3">
+        <v>2</v>
+      </c>
+      <c r="D64" s="3">
         <v>23</v>
-      </c>
-      <c r="D64" s="3">
-        <v>2302</v>
       </c>
       <c r="E64" s="3"/>
       <c r="F64" s="3" t="s">
@@ -5010,119 +5024,119 @@
       <c r="G64" s="4"/>
       <c r="H64" s="4"/>
       <c r="I64" s="4" t="s">
-        <v>75</v>
+        <v>143</v>
       </c>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A65" s="3">
-        <v>23021</v>
+        <v>2301</v>
       </c>
       <c r="B65" s="4" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="C65" s="3">
-        <v>2302</v>
+        <v>23</v>
       </c>
       <c r="D65" s="3">
-        <v>23021</v>
+        <v>2301</v>
       </c>
       <c r="E65" s="3"/>
       <c r="F65" s="3" t="s">
         <v>39</v>
       </c>
       <c r="G65" s="4" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="H65" s="4"/>
       <c r="I65" s="4" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A66" s="3">
-        <v>23022</v>
+        <v>2302</v>
       </c>
       <c r="B66" s="4" t="s">
-        <v>148</v>
+        <v>75</v>
       </c>
       <c r="C66" s="3">
+        <v>23</v>
+      </c>
+      <c r="D66" s="3">
         <v>2302</v>
-      </c>
-      <c r="D66" s="3">
-        <v>23022</v>
       </c>
       <c r="E66" s="3"/>
       <c r="F66" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="G66" s="4" t="s">
-        <v>149</v>
-      </c>
+        <v>36</v>
+      </c>
+      <c r="G66" s="4"/>
       <c r="H66" s="4"/>
       <c r="I66" s="4" t="s">
-        <v>148</v>
+        <v>75</v>
       </c>
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A67" s="3">
-        <v>2303</v>
+        <v>23021</v>
       </c>
       <c r="B67" s="4" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="C67" s="3">
-        <v>23</v>
+        <v>2302</v>
       </c>
       <c r="D67" s="3">
-        <v>2303</v>
+        <v>23021</v>
       </c>
       <c r="E67" s="3"/>
       <c r="F67" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="G67" s="4"/>
+        <v>39</v>
+      </c>
+      <c r="G67" s="4" t="s">
+        <v>147</v>
+      </c>
       <c r="H67" s="4"/>
       <c r="I67" s="4" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A68" s="3">
-        <v>23031</v>
+        <v>23022</v>
       </c>
       <c r="B68" s="4" t="s">
-        <v>65</v>
+        <v>148</v>
       </c>
       <c r="C68" s="3">
-        <v>2303</v>
+        <v>2302</v>
       </c>
       <c r="D68" s="3">
-        <v>23031</v>
+        <v>23022</v>
       </c>
       <c r="E68" s="3"/>
       <c r="F68" s="3" t="s">
         <v>39</v>
       </c>
       <c r="G68" s="4" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="H68" s="4"/>
       <c r="I68" s="4" t="s">
-        <v>65</v>
+        <v>148</v>
       </c>
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A69" s="3">
-        <v>2304</v>
+        <v>2303</v>
       </c>
       <c r="B69" s="4" t="s">
-        <v>74</v>
+        <v>150</v>
       </c>
       <c r="C69" s="3">
         <v>23</v>
       </c>
       <c r="D69" s="3">
-        <v>2304</v>
+        <v>2303</v>
       </c>
       <c r="E69" s="3"/>
       <c r="F69" s="3" t="s">
@@ -5131,465 +5145,465 @@
       <c r="G69" s="4"/>
       <c r="H69" s="4"/>
       <c r="I69" s="4" t="s">
-        <v>74</v>
+        <v>150</v>
       </c>
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A70" s="3">
-        <v>23041</v>
+        <v>23031</v>
       </c>
       <c r="B70" s="4" t="s">
-        <v>152</v>
+        <v>65</v>
       </c>
       <c r="C70" s="3">
-        <v>2304</v>
+        <v>2303</v>
       </c>
       <c r="D70" s="3">
-        <v>23041</v>
+        <v>23031</v>
       </c>
       <c r="E70" s="3"/>
       <c r="F70" s="3" t="s">
         <v>39</v>
       </c>
       <c r="G70" s="4" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="H70" s="4"/>
       <c r="I70" s="4" t="s">
-        <v>152</v>
+        <v>65</v>
       </c>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A71" s="3">
-        <v>23042</v>
+        <v>2304</v>
       </c>
       <c r="B71" s="4" t="s">
-        <v>154</v>
+        <v>74</v>
       </c>
       <c r="C71" s="3">
+        <v>23</v>
+      </c>
+      <c r="D71" s="3">
         <v>2304</v>
-      </c>
-      <c r="D71" s="3">
-        <v>23042</v>
       </c>
       <c r="E71" s="3"/>
       <c r="F71" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="G71" s="4" t="s">
-        <v>155</v>
-      </c>
+        <v>36</v>
+      </c>
+      <c r="G71" s="4"/>
       <c r="H71" s="4"/>
       <c r="I71" s="4" t="s">
-        <v>154</v>
+        <v>74</v>
       </c>
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A72" s="3">
-        <v>23043</v>
-      </c>
-      <c r="B72" s="11" t="s">
-        <v>193</v>
+        <v>23041</v>
+      </c>
+      <c r="B72" s="4" t="s">
+        <v>152</v>
       </c>
       <c r="C72" s="3">
         <v>2304</v>
       </c>
       <c r="D72" s="3">
-        <v>23043</v>
+        <v>23041</v>
       </c>
       <c r="E72" s="3"/>
       <c r="F72" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="G72" s="11" t="s">
-        <v>194</v>
+      <c r="G72" s="4" t="s">
+        <v>153</v>
       </c>
       <c r="H72" s="4"/>
-      <c r="I72" s="11" t="s">
-        <v>193</v>
+      <c r="I72" s="4" t="s">
+        <v>152</v>
       </c>
     </row>
     <row r="73" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A73" s="3">
-        <v>23044</v>
-      </c>
-      <c r="B73" s="11" t="s">
-        <v>195</v>
+        <v>23042</v>
+      </c>
+      <c r="B73" s="4" t="s">
+        <v>154</v>
       </c>
       <c r="C73" s="3">
         <v>2304</v>
       </c>
       <c r="D73" s="3">
-        <v>23044</v>
+        <v>23042</v>
       </c>
       <c r="E73" s="3"/>
       <c r="F73" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="G73" s="11" t="s">
-        <v>196</v>
+      <c r="G73" s="4" t="s">
+        <v>155</v>
       </c>
       <c r="H73" s="4"/>
-      <c r="I73" s="11" t="s">
-        <v>195</v>
+      <c r="I73" s="4" t="s">
+        <v>154</v>
       </c>
     </row>
     <row r="74" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A74" s="3">
-        <v>23045</v>
+        <v>23043</v>
       </c>
       <c r="B74" s="11" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="C74" s="3">
         <v>2304</v>
       </c>
       <c r="D74" s="3">
-        <v>23045</v>
+        <v>23043</v>
       </c>
       <c r="E74" s="3"/>
       <c r="F74" s="3" t="s">
         <v>39</v>
       </c>
       <c r="G74" s="11" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="H74" s="4"/>
       <c r="I74" s="11" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
     </row>
     <row r="75" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A75" s="3">
-        <v>23046</v>
+        <v>23044</v>
       </c>
       <c r="B75" s="11" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="C75" s="3">
         <v>2304</v>
       </c>
       <c r="D75" s="3">
-        <v>23046</v>
+        <v>23044</v>
       </c>
       <c r="E75" s="3"/>
       <c r="F75" s="3" t="s">
         <v>39</v>
       </c>
       <c r="G75" s="11" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="H75" s="4"/>
       <c r="I75" s="11" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A76" s="3">
-        <v>23047</v>
-      </c>
-      <c r="B76" s="4" t="s">
-        <v>156</v>
+        <v>23045</v>
+      </c>
+      <c r="B76" s="11" t="s">
+        <v>197</v>
       </c>
       <c r="C76" s="3">
         <v>2304</v>
       </c>
       <c r="D76" s="3">
-        <v>23047</v>
+        <v>23045</v>
       </c>
       <c r="E76" s="3"/>
       <c r="F76" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="G76" s="4" t="s">
-        <v>157</v>
+      <c r="G76" s="11" t="s">
+        <v>198</v>
       </c>
       <c r="H76" s="4"/>
-      <c r="I76" s="4" t="s">
-        <v>156</v>
+      <c r="I76" s="11" t="s">
+        <v>197</v>
       </c>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A77" s="3">
-        <v>2305</v>
-      </c>
-      <c r="B77" s="4" t="s">
-        <v>111</v>
+        <v>23046</v>
+      </c>
+      <c r="B77" s="11" t="s">
+        <v>199</v>
       </c>
       <c r="C77" s="3">
-        <v>23</v>
+        <v>2304</v>
       </c>
       <c r="D77" s="3">
-        <v>2305</v>
+        <v>23046</v>
       </c>
       <c r="E77" s="3"/>
       <c r="F77" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="G77" s="4"/>
+        <v>39</v>
+      </c>
+      <c r="G77" s="11" t="s">
+        <v>200</v>
+      </c>
       <c r="H77" s="4"/>
-      <c r="I77" s="4" t="s">
-        <v>111</v>
+      <c r="I77" s="11" t="s">
+        <v>199</v>
       </c>
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A78" s="3">
-        <v>23051</v>
+        <v>23047</v>
       </c>
       <c r="B78" s="4" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="C78" s="3">
-        <v>2305</v>
+        <v>2304</v>
       </c>
       <c r="D78" s="3">
-        <v>23051</v>
+        <v>23047</v>
       </c>
       <c r="E78" s="3"/>
       <c r="F78" s="3" t="s">
         <v>39</v>
       </c>
       <c r="G78" s="4" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="H78" s="4"/>
       <c r="I78" s="4" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
     </row>
     <row r="79" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A79" s="3">
-        <v>23052</v>
+        <v>2305</v>
       </c>
       <c r="B79" s="4" t="s">
-        <v>160</v>
+        <v>111</v>
       </c>
       <c r="C79" s="3">
+        <v>23</v>
+      </c>
+      <c r="D79" s="3">
         <v>2305</v>
-      </c>
-      <c r="D79" s="3">
-        <v>23052</v>
       </c>
       <c r="E79" s="3"/>
       <c r="F79" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="G79" s="4" t="s">
-        <v>161</v>
-      </c>
+        <v>36</v>
+      </c>
+      <c r="G79" s="4"/>
       <c r="H79" s="4"/>
       <c r="I79" s="4" t="s">
-        <v>160</v>
+        <v>111</v>
       </c>
     </row>
     <row r="80" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A80" s="3">
-        <v>23053</v>
+        <v>23051</v>
       </c>
       <c r="B80" s="4" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="C80" s="3">
         <v>2305</v>
       </c>
       <c r="D80" s="3">
-        <v>23053</v>
+        <v>23051</v>
       </c>
       <c r="E80" s="3"/>
       <c r="F80" s="3" t="s">
         <v>39</v>
       </c>
       <c r="G80" s="4" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="H80" s="4"/>
       <c r="I80" s="4" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
     </row>
     <row r="81" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A81" s="3">
-        <v>23054</v>
+        <v>23052</v>
       </c>
       <c r="B81" s="4" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="C81" s="3">
         <v>2305</v>
       </c>
       <c r="D81" s="3">
-        <v>23054</v>
+        <v>23052</v>
       </c>
       <c r="E81" s="3"/>
       <c r="F81" s="3" t="s">
         <v>39</v>
       </c>
       <c r="G81" s="4" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="H81" s="4"/>
       <c r="I81" s="4" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
     </row>
     <row r="82" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A82" s="3">
-        <v>23055</v>
+        <v>23053</v>
       </c>
       <c r="B82" s="4" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="C82" s="3">
         <v>2305</v>
       </c>
       <c r="D82" s="3">
-        <v>23055</v>
+        <v>23053</v>
       </c>
       <c r="E82" s="3"/>
       <c r="F82" s="3" t="s">
         <v>39</v>
       </c>
       <c r="G82" s="4" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="H82" s="4"/>
       <c r="I82" s="4" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
     </row>
     <row r="83" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A83" s="3">
-        <v>23056</v>
+        <v>23054</v>
       </c>
       <c r="B83" s="4" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="C83" s="3">
         <v>2305</v>
       </c>
       <c r="D83" s="3">
-        <v>23056</v>
+        <v>23054</v>
       </c>
       <c r="E83" s="3"/>
       <c r="F83" s="3" t="s">
         <v>39</v>
       </c>
       <c r="G83" s="4" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="H83" s="4"/>
       <c r="I83" s="4" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A84" s="3">
-        <v>2306</v>
+        <v>23055</v>
       </c>
       <c r="B84" s="4" t="s">
-        <v>92</v>
+        <v>166</v>
       </c>
       <c r="C84" s="3">
-        <v>23</v>
+        <v>2305</v>
       </c>
       <c r="D84" s="3">
-        <v>2306</v>
+        <v>23055</v>
       </c>
       <c r="E84" s="3"/>
       <c r="F84" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="G84" s="4"/>
+        <v>39</v>
+      </c>
+      <c r="G84" s="4" t="s">
+        <v>167</v>
+      </c>
       <c r="H84" s="4"/>
       <c r="I84" s="4" t="s">
-        <v>92</v>
+        <v>166</v>
       </c>
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A85" s="3">
-        <v>23061</v>
+        <v>23056</v>
       </c>
       <c r="B85" s="4" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="C85" s="3">
-        <v>2306</v>
+        <v>2305</v>
       </c>
       <c r="D85" s="3">
-        <v>23061</v>
+        <v>23056</v>
       </c>
       <c r="E85" s="3"/>
       <c r="F85" s="3" t="s">
         <v>39</v>
       </c>
       <c r="G85" s="4" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="H85" s="4"/>
       <c r="I85" s="4" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A86" s="3">
-        <v>24</v>
+        <v>2306</v>
       </c>
       <c r="B86" s="4" t="s">
-        <v>172</v>
+        <v>92</v>
       </c>
       <c r="C86" s="3">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="D86" s="3">
-        <v>24</v>
-      </c>
-      <c r="E86" s="4"/>
+        <v>2306</v>
+      </c>
+      <c r="E86" s="3"/>
       <c r="F86" s="3" t="s">
         <v>36</v>
       </c>
       <c r="G86" s="4"/>
       <c r="H86" s="4"/>
       <c r="I86" s="4" t="s">
-        <v>172</v>
+        <v>92</v>
       </c>
     </row>
     <row r="87" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A87" s="3">
-        <v>2401</v>
+        <v>23061</v>
       </c>
       <c r="B87" s="4" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="C87" s="3">
-        <v>24</v>
+        <v>2306</v>
       </c>
       <c r="D87" s="3">
-        <v>2401</v>
-      </c>
-      <c r="E87" s="4"/>
+        <v>23061</v>
+      </c>
+      <c r="E87" s="3"/>
       <c r="F87" s="3" t="s">
         <v>39</v>
       </c>
       <c r="G87" s="4" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="H87" s="4"/>
       <c r="I87" s="4" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A88" s="3">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B88" s="4" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="C88" s="3">
         <v>2</v>
       </c>
       <c r="D88" s="3">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E88" s="4"/>
       <c r="F88" s="3" t="s">
@@ -5598,129 +5612,177 @@
       <c r="G88" s="4"/>
       <c r="H88" s="4"/>
       <c r="I88" s="4" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
     </row>
     <row r="89" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A89" s="3">
-        <v>2501</v>
+        <v>2401</v>
       </c>
       <c r="B89" s="4" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C89" s="3">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D89" s="3">
-        <v>2501</v>
-      </c>
-      <c r="E89" s="3"/>
+        <v>2401</v>
+      </c>
+      <c r="E89" s="4"/>
       <c r="F89" s="3" t="s">
         <v>39</v>
       </c>
       <c r="G89" s="4" t="s">
-        <v>176</v>
-      </c>
-      <c r="H89" s="3"/>
+        <v>174</v>
+      </c>
+      <c r="H89" s="4"/>
       <c r="I89" s="4" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
     <row r="90" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A90" s="3">
-        <v>2502</v>
+        <v>25</v>
       </c>
       <c r="B90" s="4" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="C90" s="3">
+        <v>2</v>
+      </c>
+      <c r="D90" s="3">
         <v>25</v>
       </c>
-      <c r="D90" s="3">
-        <v>2502</v>
-      </c>
-      <c r="E90" s="3"/>
+      <c r="E90" s="4"/>
       <c r="F90" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="G90" s="4" t="s">
-        <v>178</v>
-      </c>
-      <c r="H90" s="5"/>
-      <c r="I90" s="5" t="s">
-        <v>177</v>
+        <v>36</v>
+      </c>
+      <c r="G90" s="4"/>
+      <c r="H90" s="4"/>
+      <c r="I90" s="4" t="s">
+        <v>175</v>
       </c>
     </row>
     <row r="91" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A91" s="3">
-        <v>2503</v>
+        <v>2501</v>
       </c>
       <c r="B91" s="4" t="s">
-        <v>179</v>
+        <v>172</v>
       </c>
       <c r="C91" s="3">
         <v>25</v>
       </c>
       <c r="D91" s="3">
-        <v>2503</v>
+        <v>2501</v>
       </c>
       <c r="E91" s="3"/>
       <c r="F91" s="3" t="s">
         <v>39</v>
       </c>
       <c r="G91" s="4" t="s">
-        <v>180</v>
-      </c>
-      <c r="H91" s="4"/>
+        <v>176</v>
+      </c>
+      <c r="H91" s="3"/>
       <c r="I91" s="4" t="s">
-        <v>179</v>
+        <v>172</v>
       </c>
     </row>
     <row r="92" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A92" s="3">
-        <v>26</v>
+        <v>2502</v>
       </c>
       <c r="B92" s="4" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="C92" s="3">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="D92" s="3">
-        <v>26</v>
+        <v>2502</v>
       </c>
       <c r="E92" s="3"/>
       <c r="F92" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="G92" s="4"/>
-      <c r="H92" s="4"/>
-      <c r="I92" s="4" t="s">
-        <v>181</v>
+        <v>39</v>
+      </c>
+      <c r="G92" s="4" t="s">
+        <v>178</v>
+      </c>
+      <c r="H92" s="5"/>
+      <c r="I92" s="5" t="s">
+        <v>177</v>
       </c>
     </row>
     <row r="93" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A93" s="3">
-        <v>2601</v>
+        <v>2503</v>
       </c>
       <c r="B93" s="4" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="C93" s="3">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D93" s="3">
-        <v>2601</v>
-      </c>
-      <c r="E93" s="4"/>
+        <v>2503</v>
+      </c>
+      <c r="E93" s="3"/>
       <c r="F93" s="3" t="s">
         <v>39</v>
       </c>
       <c r="G93" s="4" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="H93" s="4"/>
       <c r="I93" s="4" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="94" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A94" s="3">
+        <v>26</v>
+      </c>
+      <c r="B94" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="C94" s="3">
+        <v>2</v>
+      </c>
+      <c r="D94" s="3">
+        <v>26</v>
+      </c>
+      <c r="E94" s="3"/>
+      <c r="F94" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="G94" s="4"/>
+      <c r="H94" s="4"/>
+      <c r="I94" s="4" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="95" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A95" s="3">
+        <v>2601</v>
+      </c>
+      <c r="B95" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="C95" s="3">
+        <v>26</v>
+      </c>
+      <c r="D95" s="3">
+        <v>2601</v>
+      </c>
+      <c r="E95" s="4"/>
+      <c r="F95" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="G95" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="H95" s="4"/>
+      <c r="I95" s="4" t="s">
         <v>182</v>
       </c>
     </row>

</xml_diff>